<commit_message>
Update: Rebalancing-Tool, Obsidian workspace, .gitignore
- Rebalancing_Tool_v3.3.xlsx aktualisiert (Cowork-Session)
- .gitignore: Lock-Dateien ausgeschlossen
</commit_message>
<xml_diff>
--- a/03_Tools/Rebalancing_Tool_v3.3.xlsx
+++ b/03_Tools/Rebalancing_Tool_v3.3.xlsx
@@ -22,9 +22,12 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="185" uniqueCount="136">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="186" uniqueCount="138">
   <si>
     <t xml:space="preserve">🦅 DYNASTIE-DEPOT – Rebalancing Tool v3.3</t>
+  </si>
+  <si>
+    <t xml:space="preserve">2026-04-15</t>
   </si>
   <si>
     <t xml:space="preserve">Position</t>
@@ -148,70 +151,73 @@
     <t xml:space="preserve">AVGO</t>
   </si>
   <si>
+    <t xml:space="preserve">DEFCON 4 (86) | Insider-Check Q3</t>
+  </si>
+  <si>
+    <t xml:space="preserve">✅ Clean</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Microsoft</t>
+  </si>
+  <si>
+    <t xml:space="preserve">MSFT</t>
+  </si>
+  <si>
+    <t xml:space="preserve">DEFCON 2 (60)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">🔴 FLAG: CapEx/OCF &gt;60% | Score 60 | DEFCON 2 | Re-Check 29.04.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Costco</t>
+  </si>
+  <si>
+    <t xml:space="preserve">COST</t>
+  </si>
+  <si>
+    <t xml:space="preserve">DEFCON 4 (69) | MY 15.2% &gt; WACC</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Hermès</t>
+  </si>
+  <si>
+    <t xml:space="preserve">RMS</t>
+  </si>
+  <si>
+    <t xml:space="preserve">DEFCON 4 (71)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Veeva Systems</t>
+  </si>
+  <si>
+    <t xml:space="preserve">VEEV</t>
+  </si>
+  <si>
+    <t xml:space="preserve">DEFCON 4 (74)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Schneider Electric</t>
+  </si>
+  <si>
+    <t xml:space="preserve">SU</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Berkshire Hathaway</t>
+  </si>
+  <si>
+    <t xml:space="preserve">BRK.B</t>
+  </si>
+  <si>
+    <t xml:space="preserve">DEFCON 4 (75) | Abel Käufe $15.3M</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Visa</t>
+  </si>
+  <si>
+    <t xml:space="preserve">V</t>
+  </si>
+  <si>
     <t xml:space="preserve">DEFCON 4 (86)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">✅ Clean (Insider-Check ausstehend — OpenInsider vor Q3 FY26 Earnings prüfen)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Microsoft</t>
-  </si>
-  <si>
-    <t xml:space="preserve">MSFT</t>
-  </si>
-  <si>
-    <t xml:space="preserve">DEFCON 2 (60)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">🔴 FLAG: CapEx/OCF &gt;60% | Score 60 | DEFCON 2 | Re-Check 29.04.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Costco</t>
-  </si>
-  <si>
-    <t xml:space="preserve">COST</t>
-  </si>
-  <si>
-    <t xml:space="preserve">DEFCON 4 (~80)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">✅ Clean</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Hermès</t>
-  </si>
-  <si>
-    <t xml:space="preserve">RMS</t>
-  </si>
-  <si>
-    <t xml:space="preserve">DEFCON 4 (71)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Veeva Systems</t>
-  </si>
-  <si>
-    <t xml:space="preserve">VEEV</t>
-  </si>
-  <si>
-    <t xml:space="preserve">DEFCON 4 (74)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Schneider Electric</t>
-  </si>
-  <si>
-    <t xml:space="preserve">SU</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Berkshire Hathaway</t>
-  </si>
-  <si>
-    <t xml:space="preserve">BRK.B</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Visa</t>
-  </si>
-  <si>
-    <t xml:space="preserve">V</t>
   </si>
   <si>
     <t xml:space="preserve">Thermo Fisher</t>
@@ -1742,8 +1748,8 @@
       <c r="P1" s="2"/>
     </row>
     <row r="2" customFormat="false" ht="13.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A2" s="3" t="n">
-        <v>46127</v>
+      <c r="A2" s="3" t="s">
+        <v>1</v>
       </c>
       <c r="B2" s="3"/>
       <c r="C2" s="3"/>
@@ -1776,66 +1782,66 @@
     </row>
     <row r="4" customFormat="false" ht="36" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A4" s="5" t="s">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="B4" s="5" t="s">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="C4" s="5" t="s">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="D4" s="5" t="s">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="E4" s="5" t="s">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="F4" s="5" t="s">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="G4" s="5" t="s">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="H4" s="5" t="s">
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="I4" s="5" t="s">
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="J4" s="5" t="s">
-        <v>10</v>
+        <v>11</v>
       </c>
       <c r="K4" s="5" t="s">
-        <v>11</v>
+        <v>12</v>
       </c>
       <c r="L4" s="5" t="s">
-        <v>12</v>
+        <v>13</v>
       </c>
       <c r="M4" s="5" t="s">
-        <v>13</v>
+        <v>14</v>
       </c>
       <c r="N4" s="5" t="s">
-        <v>14</v>
+        <v>15</v>
       </c>
       <c r="O4" s="5" t="s">
-        <v>15</v>
+        <v>16</v>
       </c>
       <c r="P4" s="5" t="s">
-        <v>16</v>
+        <v>17</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="16.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A5" s="6" t="s">
-        <v>17</v>
+        <v>18</v>
       </c>
       <c r="B5" s="7" t="s">
-        <v>18</v>
+        <v>19</v>
       </c>
       <c r="C5" s="7" t="s">
-        <v>19</v>
+        <v>20</v>
       </c>
       <c r="D5" s="7" t="s">
-        <v>20</v>
+        <v>21</v>
       </c>
       <c r="E5" s="8" t="n">
         <v>0</v>
@@ -1879,16 +1885,16 @@
     </row>
     <row r="6" customFormat="false" ht="16.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A6" s="12" t="s">
-        <v>21</v>
+        <v>22</v>
       </c>
       <c r="B6" s="13" t="s">
-        <v>22</v>
+        <v>23</v>
       </c>
       <c r="C6" s="13" t="s">
-        <v>23</v>
+        <v>24</v>
       </c>
       <c r="D6" s="13" t="s">
-        <v>24</v>
+        <v>25</v>
       </c>
       <c r="E6" s="14" t="n">
         <v>0.7</v>
@@ -1932,16 +1938,16 @@
     </row>
     <row r="7" customFormat="false" ht="16.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A7" s="12" t="s">
+        <v>26</v>
+      </c>
+      <c r="B7" s="13" t="s">
+        <v>27</v>
+      </c>
+      <c r="C7" s="13" t="s">
+        <v>24</v>
+      </c>
+      <c r="D7" s="13" t="s">
         <v>25</v>
-      </c>
-      <c r="B7" s="13" t="s">
-        <v>26</v>
-      </c>
-      <c r="C7" s="13" t="s">
-        <v>23</v>
-      </c>
-      <c r="D7" s="13" t="s">
-        <v>24</v>
       </c>
       <c r="E7" s="14" t="n">
         <v>0</v>
@@ -1985,16 +1991,16 @@
     </row>
     <row r="8" customFormat="false" ht="16.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A8" s="12" t="s">
-        <v>27</v>
+        <v>28</v>
       </c>
       <c r="B8" s="13" t="s">
-        <v>28</v>
+        <v>29</v>
       </c>
       <c r="C8" s="13" t="s">
-        <v>23</v>
+        <v>24</v>
       </c>
       <c r="D8" s="13" t="s">
-        <v>24</v>
+        <v>25</v>
       </c>
       <c r="E8" s="14" t="n">
         <v>0</v>
@@ -2038,16 +2044,16 @@
     </row>
     <row r="9" customFormat="false" ht="16.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A9" s="18" t="s">
-        <v>29</v>
+        <v>30</v>
       </c>
       <c r="B9" s="19" t="s">
-        <v>30</v>
+        <v>31</v>
       </c>
       <c r="C9" s="19" t="s">
-        <v>23</v>
+        <v>24</v>
       </c>
       <c r="D9" s="19" t="s">
-        <v>20</v>
+        <v>21</v>
       </c>
       <c r="E9" s="20" t="n">
         <v>0.67</v>
@@ -2091,16 +2097,16 @@
     </row>
     <row r="10" customFormat="false" ht="16.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A10" s="24" t="s">
-        <v>31</v>
+        <v>32</v>
       </c>
       <c r="B10" s="25" t="s">
-        <v>32</v>
+        <v>33</v>
       </c>
       <c r="C10" s="25" t="s">
-        <v>33</v>
+        <v>34</v>
       </c>
       <c r="D10" s="25" t="s">
-        <v>20</v>
+        <v>21</v>
       </c>
       <c r="E10" s="26" t="n">
         <v>0</v>
@@ -2136,28 +2142,28 @@
         <v>✅ OK</v>
       </c>
       <c r="N10" s="25" t="s">
-        <v>34</v>
+        <v>35</v>
       </c>
       <c r="O10" s="25" t="s">
-        <v>35</v>
+        <v>36</v>
       </c>
       <c r="P10" s="27" t="n">
         <f aca="false">IF(C10&lt;&gt;"Aktie","",IF(LEFT(O10,1)="🔴",0,IF(LEFT(N10,8)="DEFCON 4",IF(O10="✅ Clean",('Parameter &amp; Regeln'!$B$4*'Parameter &amp; Regeln'!$B$6/(COUNTIFS($C$5:$C$20,"Aktie",$N$5:$N$20,"DEFCON 4*",$O$5:$O$20,"✅ Clean")+(COUNTIFS($C$5:$C$20,"Aktie",$N$5:$N$20,"DEFCON 3*")*'Parameter &amp; Regeln'!$B$27))),""),IF(LEFT(N10,8)="DEFCON 3",('Parameter &amp; Regeln'!$B$4*'Parameter &amp; Regeln'!$B$6*'Parameter &amp; Regeln'!$B$27/(COUNTIFS($C$5:$C$20,"Aktie",$N$5:$N$20,"DEFCON 4*",$O$5:$O$20,"✅ Clean")+(COUNTIFS($C$5:$C$20,"Aktie",$N$5:$N$20,"DEFCON 3*")*'Parameter &amp; Regeln'!$B$27))),""))))</f>
-        <v>19</v>
+        <v>16.7647058823529</v>
       </c>
     </row>
     <row r="11" customFormat="false" ht="16.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A11" s="30" t="s">
-        <v>36</v>
+        <v>37</v>
       </c>
       <c r="B11" s="31" t="s">
-        <v>37</v>
+        <v>38</v>
       </c>
       <c r="C11" s="31" t="s">
-        <v>33</v>
+        <v>34</v>
       </c>
       <c r="D11" s="31" t="s">
-        <v>20</v>
+        <v>21</v>
       </c>
       <c r="E11" s="32" t="n">
         <v>1</v>
@@ -2193,28 +2199,28 @@
         <v>✅ OK</v>
       </c>
       <c r="N11" s="31" t="s">
-        <v>38</v>
+        <v>39</v>
       </c>
       <c r="O11" s="31" t="s">
-        <v>39</v>
-      </c>
-      <c r="P11" s="33" t="str">
+        <v>40</v>
+      </c>
+      <c r="P11" s="33" t="n">
         <f aca="false">IF(C11&lt;&gt;"Aktie","",IF(LEFT(O11,1)="🔴",0,IF(LEFT(N11,8)="DEFCON 4",IF(O11="✅ Clean",('Parameter &amp; Regeln'!$B$4*'Parameter &amp; Regeln'!$B$6/(COUNTIFS($C$5:$C$20,"Aktie",$N$5:$N$20,"DEFCON 4*",$O$5:$O$20,"✅ Clean")+(COUNTIFS($C$5:$C$20,"Aktie",$N$5:$N$20,"DEFCON 3*")*'Parameter &amp; Regeln'!$B$27))),""),IF(LEFT(N11,8)="DEFCON 3",('Parameter &amp; Regeln'!$B$4*'Parameter &amp; Regeln'!$B$6*'Parameter &amp; Regeln'!$B$27/(COUNTIFS($C$5:$C$20,"Aktie",$N$5:$N$20,"DEFCON 4*",$O$5:$O$20,"✅ Clean")+(COUNTIFS($C$5:$C$20,"Aktie",$N$5:$N$20,"DEFCON 3*")*'Parameter &amp; Regeln'!$B$27))),""))))</f>
-        <v/>
+        <v>33.5294117647059</v>
       </c>
     </row>
     <row r="12" customFormat="false" ht="16.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A12" s="24" t="s">
-        <v>40</v>
+        <v>41</v>
       </c>
       <c r="B12" s="25" t="s">
-        <v>41</v>
+        <v>42</v>
       </c>
       <c r="C12" s="25" t="s">
-        <v>33</v>
+        <v>34</v>
       </c>
       <c r="D12" s="25" t="s">
-        <v>20</v>
+        <v>21</v>
       </c>
       <c r="E12" s="26" t="n">
         <v>1</v>
@@ -2250,10 +2256,10 @@
         <v>✅ OK</v>
       </c>
       <c r="N12" s="25" t="s">
-        <v>42</v>
+        <v>43</v>
       </c>
       <c r="O12" s="25" t="s">
-        <v>43</v>
+        <v>44</v>
       </c>
       <c r="P12" s="27" t="n">
         <f aca="false">IF(C12&lt;&gt;"Aktie","",IF(LEFT(O12,1)="🔴",0,IF(LEFT(N12,8)="DEFCON 4",IF(O12="✅ Clean",('Parameter &amp; Regeln'!$B$4*'Parameter &amp; Regeln'!$B$6/(COUNTIFS($C$5:$C$20,"Aktie",$N$5:$N$20,"DEFCON 4*",$O$5:$O$20,"✅ Clean")+(COUNTIFS($C$5:$C$20,"Aktie",$N$5:$N$20,"DEFCON 3*")*'Parameter &amp; Regeln'!$B$27))),""),IF(LEFT(N12,8)="DEFCON 3",('Parameter &amp; Regeln'!$B$4*'Parameter &amp; Regeln'!$B$6*'Parameter &amp; Regeln'!$B$27/(COUNTIFS($C$5:$C$20,"Aktie",$N$5:$N$20,"DEFCON 4*",$O$5:$O$20,"✅ Clean")+(COUNTIFS($C$5:$C$20,"Aktie",$N$5:$N$20,"DEFCON 3*")*'Parameter &amp; Regeln'!$B$27))),""))))</f>
@@ -2262,16 +2268,16 @@
     </row>
     <row r="13" customFormat="false" ht="16.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A13" s="30" t="s">
-        <v>44</v>
+        <v>45</v>
       </c>
       <c r="B13" s="31" t="s">
-        <v>45</v>
+        <v>46</v>
       </c>
       <c r="C13" s="31" t="s">
-        <v>33</v>
+        <v>34</v>
       </c>
       <c r="D13" s="31" t="s">
-        <v>20</v>
+        <v>21</v>
       </c>
       <c r="E13" s="32" t="n">
         <v>1</v>
@@ -2307,14 +2313,14 @@
         <v>✅ OK</v>
       </c>
       <c r="N13" s="31" t="s">
-        <v>46</v>
+        <v>47</v>
       </c>
       <c r="O13" s="31" t="s">
-        <v>47</v>
+        <v>40</v>
       </c>
       <c r="P13" s="33" t="n">
         <f aca="false">IF(C13&lt;&gt;"Aktie","",IF(LEFT(O13,1)="🔴",0,IF(LEFT(N13,8)="DEFCON 4",IF(O13="✅ Clean",('Parameter &amp; Regeln'!$B$4*'Parameter &amp; Regeln'!$B$6/(COUNTIFS($C$5:$C$20,"Aktie",$N$5:$N$20,"DEFCON 4*",$O$5:$O$20,"✅ Clean")+(COUNTIFS($C$5:$C$20,"Aktie",$N$5:$N$20,"DEFCON 3*")*'Parameter &amp; Regeln'!$B$27))),""),IF(LEFT(N13,8)="DEFCON 3",('Parameter &amp; Regeln'!$B$4*'Parameter &amp; Regeln'!$B$6*'Parameter &amp; Regeln'!$B$27/(COUNTIFS($C$5:$C$20,"Aktie",$N$5:$N$20,"DEFCON 4*",$O$5:$O$20,"✅ Clean")+(COUNTIFS($C$5:$C$20,"Aktie",$N$5:$N$20,"DEFCON 3*")*'Parameter &amp; Regeln'!$B$27))),""))))</f>
-        <v>38</v>
+        <v>33.5294117647059</v>
       </c>
     </row>
     <row r="14" customFormat="false" ht="16.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -2325,10 +2331,10 @@
         <v>49</v>
       </c>
       <c r="C14" s="25" t="s">
-        <v>33</v>
+        <v>34</v>
       </c>
       <c r="D14" s="25" t="s">
-        <v>20</v>
+        <v>21</v>
       </c>
       <c r="E14" s="26" t="n">
         <v>0</v>
@@ -2367,11 +2373,11 @@
         <v>50</v>
       </c>
       <c r="O14" s="25" t="s">
-        <v>47</v>
+        <v>40</v>
       </c>
       <c r="P14" s="27" t="n">
         <f aca="false">IF(C14&lt;&gt;"Aktie","",IF(LEFT(O14,1)="🔴",0,IF(LEFT(N14,8)="DEFCON 4",IF(O14="✅ Clean",('Parameter &amp; Regeln'!$B$4*'Parameter &amp; Regeln'!$B$6/(COUNTIFS($C$5:$C$20,"Aktie",$N$5:$N$20,"DEFCON 4*",$O$5:$O$20,"✅ Clean")+(COUNTIFS($C$5:$C$20,"Aktie",$N$5:$N$20,"DEFCON 3*")*'Parameter &amp; Regeln'!$B$27))),""),IF(LEFT(N14,8)="DEFCON 3",('Parameter &amp; Regeln'!$B$4*'Parameter &amp; Regeln'!$B$6*'Parameter &amp; Regeln'!$B$27/(COUNTIFS($C$5:$C$20,"Aktie",$N$5:$N$20,"DEFCON 4*",$O$5:$O$20,"✅ Clean")+(COUNTIFS($C$5:$C$20,"Aktie",$N$5:$N$20,"DEFCON 3*")*'Parameter &amp; Regeln'!$B$27))),""))))</f>
-        <v>38</v>
+        <v>33.5294117647059</v>
       </c>
     </row>
     <row r="15" customFormat="false" ht="16.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -2382,10 +2388,10 @@
         <v>52</v>
       </c>
       <c r="C15" s="31" t="s">
-        <v>33</v>
+        <v>34</v>
       </c>
       <c r="D15" s="31" t="s">
-        <v>20</v>
+        <v>21</v>
       </c>
       <c r="E15" s="32" t="n">
         <v>1</v>
@@ -2424,11 +2430,11 @@
         <v>53</v>
       </c>
       <c r="O15" s="31" t="s">
-        <v>47</v>
+        <v>40</v>
       </c>
       <c r="P15" s="33" t="n">
         <f aca="false">IF(C15&lt;&gt;"Aktie","",IF(LEFT(O15,1)="🔴",0,IF(LEFT(N15,8)="DEFCON 4",IF(O15="✅ Clean",('Parameter &amp; Regeln'!$B$4*'Parameter &amp; Regeln'!$B$6/(COUNTIFS($C$5:$C$20,"Aktie",$N$5:$N$20,"DEFCON 4*",$O$5:$O$20,"✅ Clean")+(COUNTIFS($C$5:$C$20,"Aktie",$N$5:$N$20,"DEFCON 3*")*'Parameter &amp; Regeln'!$B$27))),""),IF(LEFT(N15,8)="DEFCON 3",('Parameter &amp; Regeln'!$B$4*'Parameter &amp; Regeln'!$B$6*'Parameter &amp; Regeln'!$B$27/(COUNTIFS($C$5:$C$20,"Aktie",$N$5:$N$20,"DEFCON 4*",$O$5:$O$20,"✅ Clean")+(COUNTIFS($C$5:$C$20,"Aktie",$N$5:$N$20,"DEFCON 3*")*'Parameter &amp; Regeln'!$B$27))),""))))</f>
-        <v>38</v>
+        <v>33.5294117647059</v>
       </c>
     </row>
     <row r="16" customFormat="false" ht="16.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -2439,10 +2445,10 @@
         <v>55</v>
       </c>
       <c r="C16" s="25" t="s">
-        <v>33</v>
+        <v>34</v>
       </c>
       <c r="D16" s="25" t="s">
-        <v>20</v>
+        <v>21</v>
       </c>
       <c r="E16" s="26" t="n">
         <v>0</v>
@@ -2478,14 +2484,14 @@
         <v>✅ OK</v>
       </c>
       <c r="N16" s="25" t="s">
-        <v>46</v>
+        <v>50</v>
       </c>
       <c r="O16" s="25" t="s">
-        <v>47</v>
+        <v>40</v>
       </c>
       <c r="P16" s="27" t="n">
         <f aca="false">IF(C16&lt;&gt;"Aktie","",IF(LEFT(O16,1)="🔴",0,IF(LEFT(N16,8)="DEFCON 4",IF(O16="✅ Clean",('Parameter &amp; Regeln'!$B$4*'Parameter &amp; Regeln'!$B$6/(COUNTIFS($C$5:$C$20,"Aktie",$N$5:$N$20,"DEFCON 4*",$O$5:$O$20,"✅ Clean")+(COUNTIFS($C$5:$C$20,"Aktie",$N$5:$N$20,"DEFCON 3*")*'Parameter &amp; Regeln'!$B$27))),""),IF(LEFT(N16,8)="DEFCON 3",('Parameter &amp; Regeln'!$B$4*'Parameter &amp; Regeln'!$B$6*'Parameter &amp; Regeln'!$B$27/(COUNTIFS($C$5:$C$20,"Aktie",$N$5:$N$20,"DEFCON 4*",$O$5:$O$20,"✅ Clean")+(COUNTIFS($C$5:$C$20,"Aktie",$N$5:$N$20,"DEFCON 3*")*'Parameter &amp; Regeln'!$B$27))),""))))</f>
-        <v>38</v>
+        <v>33.5294117647059</v>
       </c>
     </row>
     <row r="17" customFormat="false" ht="16.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -2496,10 +2502,10 @@
         <v>57</v>
       </c>
       <c r="C17" s="31" t="s">
-        <v>33</v>
+        <v>34</v>
       </c>
       <c r="D17" s="31" t="s">
-        <v>20</v>
+        <v>21</v>
       </c>
       <c r="E17" s="32" t="n">
         <v>1</v>
@@ -2535,28 +2541,28 @@
         <v>✅ OK</v>
       </c>
       <c r="N17" s="31" t="s">
-        <v>46</v>
+        <v>58</v>
       </c>
       <c r="O17" s="31" t="s">
-        <v>47</v>
+        <v>40</v>
       </c>
       <c r="P17" s="33" t="n">
         <f aca="false">IF(C17&lt;&gt;"Aktie","",IF(LEFT(O17,1)="🔴",0,IF(LEFT(N17,8)="DEFCON 4",IF(O17="✅ Clean",('Parameter &amp; Regeln'!$B$4*'Parameter &amp; Regeln'!$B$6/(COUNTIFS($C$5:$C$20,"Aktie",$N$5:$N$20,"DEFCON 4*",$O$5:$O$20,"✅ Clean")+(COUNTIFS($C$5:$C$20,"Aktie",$N$5:$N$20,"DEFCON 3*")*'Parameter &amp; Regeln'!$B$27))),""),IF(LEFT(N17,8)="DEFCON 3",('Parameter &amp; Regeln'!$B$4*'Parameter &amp; Regeln'!$B$6*'Parameter &amp; Regeln'!$B$27/(COUNTIFS($C$5:$C$20,"Aktie",$N$5:$N$20,"DEFCON 4*",$O$5:$O$20,"✅ Clean")+(COUNTIFS($C$5:$C$20,"Aktie",$N$5:$N$20,"DEFCON 3*")*'Parameter &amp; Regeln'!$B$27))),""))))</f>
-        <v>38</v>
+        <v>33.5294117647059</v>
       </c>
     </row>
     <row r="18" customFormat="false" ht="16.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A18" s="24" t="s">
-        <v>58</v>
+        <v>59</v>
       </c>
       <c r="B18" s="25" t="s">
-        <v>59</v>
+        <v>60</v>
       </c>
       <c r="C18" s="25" t="s">
-        <v>33</v>
+        <v>34</v>
       </c>
       <c r="D18" s="25" t="s">
-        <v>20</v>
+        <v>21</v>
       </c>
       <c r="E18" s="26" t="n">
         <v>1</v>
@@ -2592,28 +2598,28 @@
         <v>✅ OK</v>
       </c>
       <c r="N18" s="25" t="s">
-        <v>46</v>
+        <v>61</v>
       </c>
       <c r="O18" s="25" t="s">
-        <v>47</v>
+        <v>40</v>
       </c>
       <c r="P18" s="27" t="n">
         <f aca="false">IF(C18&lt;&gt;"Aktie","",IF(LEFT(O18,1)="🔴",0,IF(LEFT(N18,8)="DEFCON 4",IF(O18="✅ Clean",('Parameter &amp; Regeln'!$B$4*'Parameter &amp; Regeln'!$B$6/(COUNTIFS($C$5:$C$20,"Aktie",$N$5:$N$20,"DEFCON 4*",$O$5:$O$20,"✅ Clean")+(COUNTIFS($C$5:$C$20,"Aktie",$N$5:$N$20,"DEFCON 3*")*'Parameter &amp; Regeln'!$B$27))),""),IF(LEFT(N18,8)="DEFCON 3",('Parameter &amp; Regeln'!$B$4*'Parameter &amp; Regeln'!$B$6*'Parameter &amp; Regeln'!$B$27/(COUNTIFS($C$5:$C$20,"Aktie",$N$5:$N$20,"DEFCON 4*",$O$5:$O$20,"✅ Clean")+(COUNTIFS($C$5:$C$20,"Aktie",$N$5:$N$20,"DEFCON 3*")*'Parameter &amp; Regeln'!$B$27))),""))))</f>
-        <v>38</v>
+        <v>33.5294117647059</v>
       </c>
     </row>
     <row r="19" customFormat="false" ht="16.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A19" s="30" t="s">
-        <v>60</v>
+        <v>62</v>
       </c>
       <c r="B19" s="31" t="s">
-        <v>61</v>
+        <v>63</v>
       </c>
       <c r="C19" s="31" t="s">
-        <v>33</v>
+        <v>34</v>
       </c>
       <c r="D19" s="31" t="s">
-        <v>20</v>
+        <v>21</v>
       </c>
       <c r="E19" s="32" t="n">
         <v>1</v>
@@ -2649,28 +2655,28 @@
         <v>✅ OK</v>
       </c>
       <c r="N19" s="31" t="s">
-        <v>62</v>
+        <v>64</v>
       </c>
       <c r="O19" s="31" t="s">
-        <v>63</v>
+        <v>65</v>
       </c>
       <c r="P19" s="33" t="n">
         <f aca="false">IF(C19&lt;&gt;"Aktie","",IF(LEFT(O19,1)="🔴",0,IF(LEFT(N19,8)="DEFCON 4",IF(O19="✅ Clean",('Parameter &amp; Regeln'!$B$4*'Parameter &amp; Regeln'!$B$6/(COUNTIFS($C$5:$C$20,"Aktie",$N$5:$N$20,"DEFCON 4*",$O$5:$O$20,"✅ Clean")+(COUNTIFS($C$5:$C$20,"Aktie",$N$5:$N$20,"DEFCON 3*")*'Parameter &amp; Regeln'!$B$27))),""),IF(LEFT(N19,8)="DEFCON 3",('Parameter &amp; Regeln'!$B$4*'Parameter &amp; Regeln'!$B$6*'Parameter &amp; Regeln'!$B$27/(COUNTIFS($C$5:$C$20,"Aktie",$N$5:$N$20,"DEFCON 4*",$O$5:$O$20,"✅ Clean")+(COUNTIFS($C$5:$C$20,"Aktie",$N$5:$N$20,"DEFCON 3*")*'Parameter &amp; Regeln'!$B$27))),""))))</f>
-        <v>19</v>
+        <v>16.7647058823529</v>
       </c>
     </row>
     <row r="20" customFormat="false" ht="16.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A20" s="36" t="s">
-        <v>64</v>
+        <v>66</v>
       </c>
       <c r="B20" s="37" t="s">
-        <v>65</v>
+        <v>67</v>
       </c>
       <c r="C20" s="37" t="s">
-        <v>33</v>
+        <v>34</v>
       </c>
       <c r="D20" s="37" t="s">
-        <v>20</v>
+        <v>21</v>
       </c>
       <c r="E20" s="38" t="n">
         <v>1</v>
@@ -2706,10 +2712,10 @@
         <v>✅ OK</v>
       </c>
       <c r="N20" s="37" t="s">
-        <v>66</v>
+        <v>68</v>
       </c>
       <c r="O20" s="37" t="s">
-        <v>67</v>
+        <v>69</v>
       </c>
       <c r="P20" s="39" t="n">
         <f aca="false">IF(C20&lt;&gt;"Aktie","",IF(LEFT(O20,1)="🔴",0,IF(LEFT(N20,8)="DEFCON 4",IF(O20="✅ Clean",('Parameter &amp; Regeln'!$B$4*'Parameter &amp; Regeln'!$B$6/(COUNTIFS($C$5:$C$20,"Aktie",$N$5:$N$20,"DEFCON 4*",$O$5:$O$20,"✅ Clean")+(COUNTIFS($C$5:$C$20,"Aktie",$N$5:$N$20,"DEFCON 3*")*'Parameter &amp; Regeln'!$B$27))),""),IF(LEFT(N20,8)="DEFCON 3",('Parameter &amp; Regeln'!$B$4*'Parameter &amp; Regeln'!$B$6*'Parameter &amp; Regeln'!$B$27/(COUNTIFS($C$5:$C$20,"Aktie",$N$5:$N$20,"DEFCON 4*",$O$5:$O$20,"✅ Clean")+(COUNTIFS($C$5:$C$20,"Aktie",$N$5:$N$20,"DEFCON 3*")*'Parameter &amp; Regeln'!$B$27))),""))))</f>
@@ -2718,7 +2724,7 @@
     </row>
     <row r="21" customFormat="false" ht="18.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A21" s="42" t="s">
-        <v>68</v>
+        <v>70</v>
       </c>
       <c r="B21" s="43"/>
       <c r="C21" s="43"/>
@@ -2749,7 +2755,7 @@
         <v>0.00452670992589127</v>
       </c>
       <c r="L21" s="42" t="s">
-        <v>69</v>
+        <v>71</v>
       </c>
       <c r="M21" s="47" t="n">
         <f aca="false">COUNTIF(M5:M20,"🚨 ÜBER CAP")</f>
@@ -2765,7 +2771,7 @@
       </c>
       <c r="P21" s="45" t="n">
         <f aca="false">SUMIF(C5:C20,"Aktie",P5:P20)+SUMIF(C5:C20,"&lt;&gt;Aktie",P5:P20)</f>
-        <v>931</v>
+        <v>933.235294117647</v>
       </c>
     </row>
     <row r="22" customFormat="false" ht="16.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -2784,25 +2790,25 @@
         <v>0.0320997169073292</v>
       </c>
       <c r="L22" s="54" t="s">
-        <v>70</v>
+        <v>72</v>
       </c>
       <c r="M22" s="51" t="n">
         <f aca="false">COUNTIF(M5:M9,"🚨 ÜBER CAP")</f>
         <v>0</v>
       </c>
       <c r="N22" s="49" t="s">
-        <v>71</v>
+        <v>73</v>
       </c>
       <c r="O22" s="49" t="s">
-        <v>72</v>
+        <v>74</v>
       </c>
       <c r="P22" s="55" t="s">
-        <v>73</v>
+        <v>75</v>
       </c>
     </row>
     <row r="23" customFormat="false" ht="16.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A23" s="56" t="s">
-        <v>74</v>
+        <v>76</v>
       </c>
       <c r="B23" s="57"/>
       <c r="C23" s="57"/>
@@ -2824,7 +2830,7 @@
     </row>
     <row r="24" customFormat="false" ht="16.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A24" s="62" t="s">
-        <v>75</v>
+        <v>77</v>
       </c>
       <c r="B24" s="63"/>
       <c r="C24" s="63"/>
@@ -2846,7 +2852,7 @@
     </row>
     <row r="25" customFormat="false" ht="16.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A25" s="56" t="s">
-        <v>76</v>
+        <v>78</v>
       </c>
       <c r="B25" s="57"/>
       <c r="C25" s="57"/>
@@ -2869,7 +2875,7 @@
     </row>
     <row r="26" customFormat="false" ht="16.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A26" s="62" t="s">
-        <v>77</v>
+        <v>79</v>
       </c>
       <c r="B26" s="63"/>
       <c r="C26" s="63"/>
@@ -2980,24 +2986,24 @@
   <sheetData>
     <row r="1" customFormat="false" ht="17.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A1" s="70" t="s">
-        <v>78</v>
+        <v>80</v>
       </c>
     </row>
     <row r="3" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A3" s="71" t="s">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="B3" s="71" t="s">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="C3" s="71" t="s">
-        <v>79</v>
+        <v>81</v>
       </c>
       <c r="D3" s="71" t="s">
-        <v>80</v>
+        <v>82</v>
       </c>
       <c r="E3" s="71" t="s">
-        <v>81</v>
+        <v>83</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -3354,7 +3360,7 @@
     </row>
     <row r="20" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A20" s="76" t="s">
-        <v>82</v>
+        <v>84</v>
       </c>
       <c r="C20" s="77" t="n">
         <f aca="false">'Portfolio &amp; Rebalancing'!F21</f>
@@ -3367,7 +3373,7 @@
     </row>
     <row r="22" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A22" s="76" t="s">
-        <v>83</v>
+        <v>85</v>
       </c>
       <c r="B22" s="78" t="n">
         <f aca="false">IF('Portfolio &amp; Rebalancing'!F25=0,0,E20/'Portfolio &amp; Rebalancing'!F25)</f>
@@ -3376,7 +3382,7 @@
     </row>
     <row r="23" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A23" s="76" t="s">
-        <v>84</v>
+        <v>86</v>
       </c>
       <c r="B23" s="78" t="n">
         <f aca="false">SUMPRODUCT('Portfolio &amp; Rebalancing'!$E$5:$E$20,'Portfolio &amp; Rebalancing'!$I$5:$I$20)/SUM('Portfolio &amp; Rebalancing'!$I$5:$I$20)</f>
@@ -3385,7 +3391,7 @@
     </row>
     <row r="24" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A24" s="76" t="s">
-        <v>85</v>
+        <v>87</v>
       </c>
       <c r="B24" s="79" t="n">
         <f aca="false">'Parameter &amp; Regeln'!B11</f>
@@ -3394,7 +3400,7 @@
     </row>
     <row r="25" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A25" s="76" t="s">
-        <v>86</v>
+        <v>88</v>
       </c>
       <c r="B25" s="76" t="str">
         <f aca="false">IF(B22&gt;B24,"⛔ ÜBER CAP","✅ OK")</f>
@@ -3403,7 +3409,7 @@
     </row>
     <row r="26" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A26" s="76" t="s">
-        <v>87</v>
+        <v>89</v>
       </c>
       <c r="B26" s="80" t="str">
         <f aca="false">IF(B23&gt;B24,"⛔ ZIEL ÜBER CAP","✅ Ziel OK")</f>
@@ -3437,111 +3443,111 @@
   <sheetData>
     <row r="1" customFormat="false" ht="17.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A1" s="70" t="s">
-        <v>88</v>
+        <v>90</v>
       </c>
     </row>
     <row r="3" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A3" s="71" t="s">
-        <v>89</v>
+        <v>91</v>
       </c>
       <c r="B3" s="71" t="s">
-        <v>90</v>
+        <v>92</v>
       </c>
       <c r="C3" s="71" t="s">
-        <v>91</v>
+        <v>93</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A4" s="72" t="s">
-        <v>92</v>
+        <v>94</v>
       </c>
       <c r="B4" s="81" t="n">
         <v>950</v>
       </c>
       <c r="C4" s="82" t="s">
-        <v>93</v>
+        <v>95</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A5" s="72" t="s">
-        <v>94</v>
+        <v>96</v>
       </c>
       <c r="B5" s="83" t="n">
         <v>0.65</v>
       </c>
       <c r="C5" s="82" t="s">
-        <v>95</v>
+        <v>97</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A6" s="72" t="s">
-        <v>96</v>
+        <v>98</v>
       </c>
       <c r="B6" s="83" t="n">
         <v>0.3</v>
       </c>
       <c r="C6" s="82" t="s">
-        <v>95</v>
+        <v>97</v>
       </c>
     </row>
     <row r="7" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A7" s="72" t="s">
-        <v>97</v>
+        <v>99</v>
       </c>
       <c r="B7" s="83" t="n">
         <v>0.05</v>
       </c>
       <c r="C7" s="82" t="s">
-        <v>95</v>
+        <v>97</v>
       </c>
     </row>
     <row r="8" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A8" s="72" t="s">
-        <v>98</v>
+        <v>100</v>
       </c>
       <c r="B8" s="84" t="n">
         <v>0.015</v>
       </c>
       <c r="C8" s="82" t="s">
-        <v>95</v>
+        <v>97</v>
       </c>
     </row>
     <row r="9" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A9" s="85" t="s">
-        <v>99</v>
+        <v>101</v>
       </c>
       <c r="B9" s="86" t="n">
         <v>0.04</v>
       </c>
       <c r="C9" s="87" t="s">
-        <v>95</v>
+        <v>97</v>
       </c>
     </row>
     <row r="10" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A10" s="72" t="s">
-        <v>100</v>
+        <v>102</v>
       </c>
       <c r="B10" s="83" t="n">
         <v>0.1</v>
       </c>
       <c r="C10" s="82" t="s">
-        <v>95</v>
+        <v>97</v>
       </c>
     </row>
     <row r="11" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A11" s="72" t="s">
-        <v>85</v>
+        <v>87</v>
       </c>
       <c r="B11" s="83" t="n">
         <v>0.63</v>
       </c>
       <c r="C11" s="82" t="s">
-        <v>95</v>
+        <v>97</v>
       </c>
     </row>
     <row r="12" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A12" s="72" t="s">
-        <v>101</v>
+        <v>103</v>
       </c>
       <c r="B12" s="82" t="n">
         <v>11</v>
@@ -3550,7 +3556,7 @@
     </row>
     <row r="13" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A13" s="72" t="s">
-        <v>102</v>
+        <v>104</v>
       </c>
       <c r="B13" s="82" t="n">
         <f aca="false">COUNTIF('Portfolio &amp; Rebalancing'!C5:C20,"Aktie")</f>
@@ -3560,7 +3566,7 @@
     </row>
     <row r="14" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A14" s="88" t="s">
-        <v>103</v>
+        <v>105</v>
       </c>
       <c r="B14" s="89" t="n">
         <f aca="false">COUNTA('Portfolio &amp; Rebalancing'!A5:A20)</f>
@@ -3569,168 +3575,168 @@
     </row>
     <row r="15" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A15" s="90" t="s">
-        <v>104</v>
+        <v>106</v>
       </c>
       <c r="B15" s="87" t="n">
         <v>0.15</v>
       </c>
       <c r="C15" s="91" t="s">
-        <v>95</v>
+        <v>97</v>
       </c>
     </row>
     <row r="16" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A16" s="90" t="s">
-        <v>105</v>
+        <v>107</v>
       </c>
       <c r="B16" s="92" t="n">
         <f aca="false">B5+B6+B7</f>
         <v>1</v>
       </c>
       <c r="C16" s="91" t="s">
-        <v>95</v>
+        <v>97</v>
       </c>
     </row>
     <row r="17" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A17" s="93" t="s">
-        <v>106</v>
+        <v>108</v>
       </c>
     </row>
     <row r="18" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
     <row r="19" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A19" s="94" t="s">
-        <v>107</v>
+        <v>109</v>
       </c>
       <c r="B19" s="94" t="s">
-        <v>108</v>
+        <v>110</v>
       </c>
       <c r="C19" s="94" t="s">
-        <v>12</v>
+        <v>13</v>
       </c>
     </row>
     <row r="20" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A20" s="72" t="s">
-        <v>109</v>
+        <v>111</v>
       </c>
       <c r="B20" s="82" t="s">
-        <v>110</v>
+        <v>112</v>
       </c>
       <c r="C20" s="82" t="s">
-        <v>111</v>
+        <v>113</v>
       </c>
     </row>
     <row r="21" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A21" s="72" t="s">
-        <v>112</v>
+        <v>114</v>
       </c>
       <c r="B21" s="82" t="s">
-        <v>113</v>
+        <v>115</v>
       </c>
       <c r="C21" s="82" t="s">
-        <v>114</v>
+        <v>116</v>
       </c>
     </row>
     <row r="22" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A22" s="72" t="s">
-        <v>115</v>
+        <v>117</v>
       </c>
       <c r="B22" s="82" t="s">
-        <v>116</v>
+        <v>118</v>
       </c>
       <c r="C22" s="82" t="s">
-        <v>117</v>
+        <v>119</v>
       </c>
     </row>
     <row r="23" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A23" s="72" t="s">
-        <v>118</v>
+        <v>120</v>
       </c>
       <c r="B23" s="82" t="s">
-        <v>119</v>
+        <v>121</v>
       </c>
       <c r="C23" s="82" t="s">
-        <v>120</v>
+        <v>122</v>
       </c>
     </row>
     <row r="25" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A25" s="95" t="s">
-        <v>121</v>
+        <v>123</v>
       </c>
       <c r="B25" s="96" t="n">
         <f aca="false">B4*B6</f>
         <v>285</v>
       </c>
       <c r="C25" s="97" t="s">
-        <v>93</v>
+        <v>95</v>
       </c>
     </row>
     <row r="26" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A26" s="95" t="s">
-        <v>122</v>
+        <v>124</v>
       </c>
       <c r="B26" s="98" t="n">
         <f aca="false">COUNTIFS('Portfolio &amp; Rebalancing'!$C$10:$C$20,"Aktie",'Portfolio &amp; Rebalancing'!$N$10:$N$20,"DEFCON 4*",'Portfolio &amp; Rebalancing'!$O$10:$O$20,"✅ Clean")</f>
-        <v>6</v>
+        <v>7</v>
       </c>
     </row>
     <row r="27" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A27" s="99" t="s">
-        <v>123</v>
+        <v>125</v>
       </c>
       <c r="B27" s="100" t="n">
         <v>0.5</v>
       </c>
       <c r="C27" s="99" t="s">
-        <v>95</v>
+        <v>97</v>
       </c>
     </row>
     <row r="28" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A28" s="101" t="s">
-        <v>124</v>
+        <v>126</v>
       </c>
     </row>
     <row r="29" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A29" s="99" t="s">
-        <v>125</v>
+        <v>127</v>
       </c>
       <c r="B29" s="102" t="s">
-        <v>126</v>
+        <v>128</v>
       </c>
       <c r="C29" s="99" t="s">
-        <v>127</v>
+        <v>129</v>
       </c>
     </row>
     <row r="30" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A30" s="99" t="s">
-        <v>128</v>
+        <v>130</v>
       </c>
       <c r="B30" s="102" t="s">
-        <v>129</v>
+        <v>131</v>
       </c>
       <c r="C30" s="99" t="s">
-        <v>130</v>
+        <v>132</v>
       </c>
     </row>
     <row r="31" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A31" s="99" t="s">
-        <v>131</v>
+        <v>133</v>
       </c>
       <c r="B31" s="102" t="s">
-        <v>132</v>
+        <v>134</v>
       </c>
       <c r="C31" s="99" t="s">
-        <v>133</v>
+        <v>135</v>
       </c>
     </row>
     <row r="32" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A32" s="99" t="s">
-        <v>134</v>
+        <v>136</v>
       </c>
       <c r="B32" s="102" t="n">
         <f aca="false">B4*B6/(COUNTIFS('Portfolio &amp; Rebalancing'!$C$10:$C$20,"Aktie",'Portfolio &amp; Rebalancing'!$N$10:$N$20,"DEFCON 4*",'Portfolio &amp; Rebalancing'!$O$10:$O$20,"✅ Clean")+(COUNTIFS('Portfolio &amp; Rebalancing'!$C$10:$C$20,"Aktie",'Portfolio &amp; Rebalancing'!$N$10:$N$20,"DEFCON 3*")*B27))</f>
-        <v>38</v>
+        <v>33.5294117647059</v>
       </c>
       <c r="C32" s="99" t="s">
-        <v>135</v>
+        <v>137</v>
       </c>
     </row>
   </sheetData>

</xml_diff>